<commit_message>
fix delivery entry and add a queue module desktop alert
</commit_message>
<xml_diff>
--- a/public/templates/IAR-2025.xlsx
+++ b/public/templates/IAR-2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\NIA-PROJECT\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\AIMS\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1041606-A8D4-4CEC-9184-B78A7BCF2F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36AD6B3C-F0B7-4517-A014-EDF07E2C0856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
   <si>
     <t>Entity Name:</t>
   </si>
@@ -156,12 +156,6 @@
     <t>Procurement Analyst B</t>
   </si>
   <si>
-    <t>Functionality</t>
-  </si>
-  <si>
-    <t>Specifications</t>
-  </si>
-  <si>
     <t>Date of Acceptance:</t>
   </si>
   <si>
@@ -175,6 +169,15 @@
   </si>
   <si>
     <t>NIA ACIMO -</t>
+  </si>
+  <si>
+    <t>Quantity:</t>
+  </si>
+  <si>
+    <t>Specifications:</t>
+  </si>
+  <si>
+    <t>Functionality:</t>
   </si>
 </sst>
 </file>
@@ -768,7 +771,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="6" applyFont="1"/>
@@ -894,15 +897,118 @@
     <xf numFmtId="43" fontId="8" fillId="0" borderId="27" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="33" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -963,113 +1069,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="33" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1253,7 +1257,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>56842</xdr:colOff>
+      <xdr:colOff>56843</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>634407</xdr:rowOff>
     </xdr:to>
@@ -1314,7 +1318,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>915035</xdr:colOff>
+      <xdr:colOff>915036</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>27938</xdr:rowOff>
     </xdr:to>
@@ -1412,7 +1416,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>384674</xdr:colOff>
+      <xdr:colOff>241799</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>639181</xdr:rowOff>
     </xdr:to>
@@ -1748,9 +1752,9 @@
   <cols>
     <col min="1" max="1" width="9.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="2.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="2.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="42.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.28515625" style="1" customWidth="1"/>
     <col min="8" max="8" width="2.7109375" style="1" customWidth="1"/>
@@ -2212,15 +2216,15 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="94" t="s">
+      <c r="F2" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
     </row>
     <row r="3" spans="1:13" s="2" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:13" s="5" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2228,29 +2232,29 @@
         <v>0</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="C4" s="95" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="95"/>
-      <c r="J4" s="95"/>
-      <c r="K4" s="95"/>
-      <c r="L4" s="95"/>
-      <c r="M4" s="95"/>
+      <c r="C4" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
     </row>
     <row r="5" spans="1:13" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="106" t="s">
+      <c r="A5" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="107"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -2262,15 +2266,15 @@
       <c r="M5" s="48"/>
     </row>
     <row r="6" spans="1:13" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="74" t="s">
+      <c r="A6" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="73"/>
       <c r="C6" s="38"/>
-      <c r="D6" s="51" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="51"/>
+      <c r="D6" s="87" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="87"/>
       <c r="F6" s="42"/>
       <c r="L6" s="8" t="s">
         <v>5</v>
@@ -2278,15 +2282,15 @@
       <c r="M6" s="44"/>
     </row>
     <row r="7" spans="1:13" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="74" t="s">
+      <c r="A7" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="109" t="s">
-        <v>46</v>
-      </c>
-      <c r="E7" s="109"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="75" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="75"/>
       <c r="F7" s="9"/>
       <c r="L7" s="4" t="s">
         <v>19</v>
@@ -2294,13 +2298,13 @@
       <c r="M7" s="45"/>
     </row>
     <row r="8" spans="1:13" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
+      <c r="B8" s="73"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="109"/>
+      <c r="E8" s="109"/>
       <c r="F8" s="9"/>
       <c r="L8" s="4" t="s">
         <v>5</v>
@@ -2308,22 +2312,22 @@
       <c r="M8" s="46"/>
     </row>
     <row r="9" spans="1:13" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="74" t="s">
+      <c r="A9" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="75"/>
-      <c r="D9" s="71"/>
-      <c r="E9" s="71"/>
-      <c r="F9" s="71"/>
+      <c r="B9" s="73"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="106"/>
+      <c r="F9" s="106"/>
       <c r="L9" s="4" t="s">
         <v>21</v>
       </c>
       <c r="M9" s="45"/>
     </row>
     <row r="10" spans="1:13" s="5" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="72"/>
-      <c r="B10" s="73"/>
+      <c r="A10" s="107"/>
+      <c r="B10" s="108"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
@@ -2348,27 +2352,27 @@
       <c r="K11" s="15"/>
     </row>
     <row r="12" spans="1:13" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="103" t="s">
+      <c r="A12" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="52" t="s">
+      <c r="B12" s="67"/>
+      <c r="C12" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="58"/>
-      <c r="E12" s="53"/>
+      <c r="D12" s="93"/>
+      <c r="E12" s="67"/>
       <c r="F12" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="52" t="s">
+      <c r="G12" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="H12" s="53"/>
-      <c r="I12" s="52" t="s">
+      <c r="H12" s="67"/>
+      <c r="I12" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="J12" s="58"/>
-      <c r="K12" s="53"/>
+      <c r="J12" s="93"/>
+      <c r="K12" s="67"/>
       <c r="L12" s="16" t="s">
         <v>25</v>
       </c>
@@ -2377,38 +2381,38 @@
       </c>
     </row>
     <row r="13" spans="1:13" s="2" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="104"/>
-      <c r="B13" s="105"/>
-      <c r="C13" s="66"/>
-      <c r="D13" s="67"/>
-      <c r="E13" s="68"/>
+      <c r="A13" s="68"/>
+      <c r="B13" s="69"/>
+      <c r="C13" s="101"/>
+      <c r="D13" s="102"/>
+      <c r="E13" s="103"/>
       <c r="F13" s="18"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="60"/>
-      <c r="K13" s="61"/>
+      <c r="G13" s="89"/>
+      <c r="H13" s="90"/>
+      <c r="I13" s="94"/>
+      <c r="J13" s="95"/>
+      <c r="K13" s="96"/>
       <c r="L13" s="49"/>
       <c r="M13" s="50"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="96" t="s">
+      <c r="A14" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="97"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98" t="s">
+      <c r="B14" s="60"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="98"/>
-      <c r="I14" s="98"/>
-      <c r="J14" s="98"/>
-      <c r="K14" s="98"/>
-      <c r="L14" s="98"/>
-      <c r="M14" s="99"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
+      <c r="M14" s="62"/>
     </row>
     <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
@@ -2421,44 +2425,44 @@
       <c r="F15" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="G15" s="100" t="s">
+      <c r="G15" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="101"/>
-      <c r="I15" s="101"/>
-      <c r="J15" s="101"/>
-      <c r="K15" s="101"/>
-      <c r="L15" s="101"/>
-      <c r="M15" s="102"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="64"/>
+      <c r="J15" s="64"/>
+      <c r="K15" s="64"/>
+      <c r="L15" s="64"/>
+      <c r="M15" s="65"/>
     </row>
     <row r="16" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="69" t="s">
+      <c r="A16" s="104" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="64"/>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="64"/>
-      <c r="F16" s="70"/>
+      <c r="B16" s="99"/>
+      <c r="C16" s="99"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="105"/>
       <c r="G16" s="43" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H16" s="36"/>
       <c r="I16" s="36"/>
-      <c r="J16" s="64"/>
-      <c r="K16" s="64"/>
-      <c r="L16" s="64"/>
-      <c r="M16" s="65"/>
+      <c r="J16" s="99"/>
+      <c r="K16" s="99"/>
+      <c r="L16" s="99"/>
+      <c r="M16" s="100"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="22"/>
       <c r="B17" s="36"/>
       <c r="C17" s="23"/>
       <c r="D17" s="41"/>
-      <c r="E17" s="83" t="s">
+      <c r="E17" s="81" t="s">
         <v>34</v>
       </c>
-      <c r="F17" s="84"/>
+      <c r="F17" s="82"/>
       <c r="G17" s="43"/>
       <c r="H17" s="36"/>
       <c r="I17" s="36"/>
@@ -2469,79 +2473,79 @@
     </row>
     <row r="18" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="24"/>
-      <c r="B18" s="39"/>
+      <c r="B18" s="110"/>
       <c r="C18" s="25" t="s">
         <v>33</v>
       </c>
       <c r="D18" s="25"/>
-      <c r="E18" s="83"/>
-      <c r="F18" s="84"/>
+      <c r="E18" s="81"/>
+      <c r="F18" s="82"/>
       <c r="G18" s="26"/>
       <c r="H18" s="39"/>
       <c r="I18" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="J18" s="62"/>
-      <c r="K18" s="63"/>
-      <c r="L18" s="56" t="s">
-        <v>43</v>
-      </c>
-      <c r="M18" s="57"/>
+      <c r="J18" s="97"/>
+      <c r="K18" s="98"/>
+      <c r="L18" s="91" t="s">
+        <v>41</v>
+      </c>
+      <c r="M18" s="92"/>
     </row>
     <row r="19" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="24"/>
-      <c r="B19" s="39"/>
+      <c r="B19" s="110"/>
       <c r="C19" s="25" t="s">
         <v>35</v>
       </c>
       <c r="D19" s="40"/>
-      <c r="E19" s="81" t="s">
-        <v>2</v>
-      </c>
-      <c r="F19" s="82"/>
+      <c r="E19" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="F19" s="51"/>
       <c r="G19" s="26"/>
       <c r="H19" s="37"/>
       <c r="I19" s="25"/>
       <c r="J19" s="25"/>
       <c r="K19" s="25"/>
-      <c r="L19" s="87"/>
-      <c r="M19" s="88"/>
+      <c r="L19" s="85"/>
+      <c r="M19" s="86"/>
     </row>
     <row r="20" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="24"/>
-      <c r="B20" s="39"/>
+      <c r="B20" s="110"/>
       <c r="C20" s="25" t="s">
         <v>36</v>
       </c>
       <c r="D20" s="40"/>
-      <c r="E20" s="81" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20" s="82"/>
+      <c r="E20" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="51"/>
       <c r="G20" s="28"/>
       <c r="H20" s="23"/>
       <c r="I20" s="23"/>
       <c r="J20" s="23"/>
       <c r="K20" s="23"/>
-      <c r="L20" s="85"/>
-      <c r="M20" s="86"/>
+      <c r="L20" s="83"/>
+      <c r="M20" s="84"/>
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="24"/>
       <c r="B21" s="37"/>
       <c r="C21" s="25"/>
       <c r="D21" s="40"/>
-      <c r="E21" s="81" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" s="82"/>
+      <c r="E21" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" s="51"/>
       <c r="G21" s="28"/>
       <c r="H21" s="23"/>
       <c r="I21" s="23"/>
       <c r="J21" s="23"/>
       <c r="K21" s="23"/>
-      <c r="L21" s="85"/>
-      <c r="M21" s="86"/>
+      <c r="L21" s="83"/>
+      <c r="M21" s="84"/>
     </row>
     <row r="22" spans="1:13" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A22" s="24"/>
@@ -2608,23 +2612,23 @@
       <c r="M25" s="80"/>
     </row>
     <row r="26" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="89" t="s">
+      <c r="A26" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="90"/>
-      <c r="C26" s="90"/>
-      <c r="D26" s="90"/>
-      <c r="E26" s="90"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="91" t="s">
+      <c r="B26" s="53"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="H26" s="92"/>
-      <c r="I26" s="92"/>
-      <c r="J26" s="92"/>
-      <c r="K26" s="92"/>
-      <c r="L26" s="92"/>
-      <c r="M26" s="93"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="55"/>
+      <c r="K26" s="55"/>
+      <c r="L26" s="55"/>
+      <c r="M26" s="56"/>
     </row>
     <row r="28" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2699,7 +2703,27 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="36">
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J16:M16"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="G25:M25"/>
+    <mergeCell ref="E17:F18"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="G26:M26"/>
     <mergeCell ref="F2:L2"/>
@@ -2715,33 +2739,11 @@
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="D7:E7"/>
-    <mergeCell ref="E19:F19"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="G25:M25"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E17:F18"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J16:M16"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A9:C9"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.196850393700787" right="0" top="0.761811024" bottom="0.511811023622047" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup scale="78" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="75" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>